<commit_message>
chore: snapshot before cleanup (safety net)
</commit_message>
<xml_diff>
--- a/outputs/019f7e48-3b54-7983-8b02-5f8cc68fafd6/稲敷市・美浦村.xlsx
+++ b/outputs/019f7e48-3b54-7983-8b02-5f8cc68fafd6/稲敷市・美浦村.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_カフェ" sheetId="1" r:id="R3a15b220cdef431f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_居酒屋" sheetId="2" r:id="R3c7e30d0c47d4206"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_スナック" sheetId="3" r:id="R475e5369cfbe4330"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_パン屋" sheetId="4" r:id="R7e2770abc7514f3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_スイーツ" sheetId="5" r:id="R360a7f938b264fcd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_和食" sheetId="6" r:id="R94a62284da694117"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_定食・食堂" sheetId="7" r:id="R367820d1cce94d16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_韓国" sheetId="8" r:id="Rc7644785cef14add"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_ラーメン" sheetId="9" r:id="Rdd067c752cc44a64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_Bar" sheetId="10" r:id="Rc41234c8c5f44fe1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_焼き鳥" sheetId="11" r:id="R3b654a1350d34978"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_お好み焼き" sheetId="12" r:id="R9bc6db4ba20c4ed7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_焼肉" sheetId="13" r:id="Rb78c8147dda44f57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_中華" sheetId="14" r:id="R62fed201b0fe4e39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_蕎麦・うどん" sheetId="15" r:id="Raac536b41b0849cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_寿司" sheetId="16" r:id="R8a5a8045b9d34054"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_洋食" sheetId="17" r:id="Ree0013afe6e54e0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_テイクアウト専門店" sheetId="18" r:id="Rad78e09bb86942be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_カフェ" sheetId="1" r:id="Rf9f209e6ef6746dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_居酒屋" sheetId="2" r:id="R4962619da9534679"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_スナック" sheetId="3" r:id="Rfb7cb98448924d58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_パン屋" sheetId="4" r:id="R31983f240b9740c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_スイーツ" sheetId="5" r:id="R9ad88a91ed7f49b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_和食" sheetId="6" r:id="R522a4d45ae4e4f3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_定食・食堂" sheetId="7" r:id="Ra4452d371de844ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_韓国" sheetId="8" r:id="Rce043db5bf7b4627"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_ラーメン" sheetId="9" r:id="R387c2045e73e4434"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_Bar" sheetId="10" r:id="R65c0f431dbfc4b6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_焼き鳥" sheetId="11" r:id="R3416a217f87f4e02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_お好み焼き" sheetId="12" r:id="Rd617657fb8dc4473"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_焼肉" sheetId="13" r:id="R04cd3f54526a4a0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_中華" sheetId="14" r:id="R7329b16bd27a4cdf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_蕎麦・うどん" sheetId="15" r:id="Rdbeb977f98da4d65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_寿司" sheetId="16" r:id="Ra9c0a6219bcd4a7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_洋食" sheetId="17" r:id="R3b005f6bd2b34b46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SALES_テイクアウト専門店" sheetId="18" r:id="Rab268cae538f4a66"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>